<commit_message>
Update Kumu database description, add v1 tag and add a reference for metathesis reaction with a pathway via butane.
</commit_message>
<xml_diff>
--- a/Kumu_data/kumu-nicolas-lienart-screenlca-paper-biobased-pathways.xlsx
+++ b/Kumu_data/kumu-nicolas-lienart-screenlca-paper-biobased-pathways.xlsx
@@ -4637,7 +4637,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>(Zacharopoulou and Lemonidou, 2018; Wang et al., 2020)</t>
+          <t>(Zacharopoulou and Lemonidou, 2018; Wang et al., 2020; Kikuchi et al., 2017)</t>
         </is>
       </c>
     </row>
@@ -5716,6 +5716,30 @@
       <c r="L248" t="inlineStr">
         <is>
           <t>(Sardon et al., 2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Dimerization of ethylene to butane</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>(Kikuchi et al., 2017)</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Butane</t>
         </is>
       </c>
     </row>
@@ -11557,6 +11581,57 @@
         </is>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Ethylene</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Dimerization of ethylene to butane</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>directed</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Dimerization of ethylene to butane</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Butane</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>directed</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Butane</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Metathesis to propylene</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>directed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>